<commit_message>
Research Methodology Folders added
</commit_message>
<xml_diff>
--- a/research/RP-001_Rockefeller_Methodology/WASHINGTON_2020_LEDGER.xlsx
+++ b/research/RP-001_Rockefeller_Methodology/WASHINGTON_2020_LEDGER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\washington-county-federal-fiscal-balance\research\RP-001_Rockefeller_Methodology\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3674E1E8-01F9-4DFD-A330-36DE185A3D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D77326-E697-4FDF-BA2F-D30C7DC1A78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E653176B-D3C8-43EA-B770-03F880A93C8A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E653176B-D3C8-43EA-B770-03F880A93C8A}"/>
   </bookViews>
   <sheets>
     <sheet name="01 Summary" sheetId="6" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
   <si>
     <t>Metric</t>
   </si>
@@ -158,6 +158,33 @@
   </si>
   <si>
     <t>COVID Programs</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Citation</t>
+  </si>
+  <si>
+    <t>Uses IRS SOI tax liability allocation rather than IRS Table 5 gross collections</t>
+  </si>
+  <si>
+    <t>R25-IIT</t>
+  </si>
+  <si>
+    <t>Uses BEA allocation methodology</t>
+  </si>
+  <si>
+    <t>R25-CORP</t>
+  </si>
+  <si>
+    <t>Overall Methodology</t>
+  </si>
+  <si>
+    <t>Rockefeller allocates national receipt categories to states</t>
+  </si>
+  <si>
+    <t>R25-METH-ALLOC</t>
   </si>
 </sst>
 </file>
@@ -656,7 +683,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FEFAC0A-3717-4B20-9A6B-BF8DCED51C7B}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.5703125" customWidth="1"/>
@@ -665,9 +692,11 @@
     <col min="4" max="4" width="28.28515625" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" customWidth="1"/>
     <col min="6" max="6" width="27.5703125" customWidth="1"/>
+    <col min="7" max="7" width="52.42578125" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -686,8 +715,14 @@
       <c r="F1" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>18</v>
       </c>
@@ -698,8 +733,14 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -710,8 +751,14 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -723,7 +770,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -735,7 +782,7 @@
       <c r="E5" s="3"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>26</v>
       </c>
@@ -746,6 +793,17 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>